<commit_message>
Marcar entre corchetes los datos pendientes (ANMAC, lote, manzana, calle, fechas) y cargar el contacto en las planillas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JmsTv5NfzGveoXYqHYwuQV
</commit_message>
<xml_diff>
--- a/XANTRAX_Pedido_Cotizacion_Proveedores.xlsx
+++ b/XANTRAX_Pedido_Cotizacion_Proveedores.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Lote / manzana</t>
   </si>
   <si>
-    <t xml:space="preserve">[____]</t>
+    <t xml:space="preserve">Lote [N° de lote], manzana [N° de manzana]</t>
   </si>
   <si>
     <t xml:space="preserve">Datos del proveedor (completar)</t>
@@ -43,7 +43,7 @@
     <t xml:space="preserve">Contacto para consultas</t>
   </si>
   <si>
-    <t xml:space="preserve">[nombre, teléfono, correo]</t>
+    <t xml:space="preserve">Ignacio Ramallo, socio gerente · +54 9 299 467-5788 · iramallo@xantrax.com.ar</t>
   </si>
   <si>
     <t xml:space="preserve">Razón social</t>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Fecha límite de respuesta</t>
   </si>
   <si>
-    <t xml:space="preserve">[__/__/2026]</t>
+    <t xml:space="preserve">[fecha límite de respuesta]</t>
   </si>
   <si>
     <t xml:space="preserve">CUIT</t>

</xml_diff>